<commit_message>
feat: add tkinter GUI and improve failure handling
- Add full Tkinter GUI application with tabs for student registration and medical scanning, including file browsing, school/class selection, and async job logging.
- Refactor main.py and scanning.py to use modular run functions, switch to Chrome webdriver, and remove hardcoded paths/credentials.
- Implement robust failure tracking: collect failed submissions, export timestamped Excel/TXT logs to user's Downloads, and update failed_names.txt.
- Overhaul ui.py with complete school database, updated XPath selectors, and dynamic school/class selection helpers.
- Rewrite form submission logic to handle errors gracefully and log failed entries.
- Update input Excel files and failed_names.txt with latest test data.
</commit_message>
<xml_diff>
--- a/PEMERIKSAAN KLS 6.xlsx
+++ b/PEMERIKSAAN KLS 6.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SD\SD BOJONGASIH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SD\SDN 3 BOJONGASIH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE485035-4E39-44DD-8EB8-F3C034A49196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFA41EE1-0970-4695-95E8-81BC1C1DBC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{A2C7ED5D-0953-4269-B868-BC3D5FA083FB}"/>
   </bookViews>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>nama</t>
   </si>
@@ -93,88 +96,37 @@
     <t>tm 11</t>
   </si>
   <si>
-    <t>ALPAHRI MUHAMAD YUSUF</t>
-  </si>
-  <si>
-    <t>BELLA TIARA SUTISNA</t>
-  </si>
-  <si>
-    <t>DIANDRA ABDUL ROHMAN</t>
-  </si>
-  <si>
-    <t>FIKI ZAENAL ALI</t>
-  </si>
-  <si>
-    <t>MUHAMAD FUADUL MU'JIB</t>
-  </si>
-  <si>
-    <t>MUHAMMAD KAMIL PASYA</t>
-  </si>
-  <si>
-    <t>NAJMA SHIDQIYYA</t>
-  </si>
-  <si>
-    <t>RAISYA NURPADILAH</t>
-  </si>
-  <si>
-    <t>RAZWA NURUL DZIHNI</t>
-  </si>
-  <si>
-    <t>REIHAN AFANDI YANWAR</t>
-  </si>
-  <si>
-    <t>RINTA SINTIA RAHAYU</t>
-  </si>
-  <si>
-    <t>SANDRA DRUPADI</t>
-  </si>
-  <si>
-    <t>SINVIA NUR SA ADAH</t>
-  </si>
-  <si>
-    <t>TRIAS HIJA FAHRANI</t>
-  </si>
-  <si>
-    <t>ZIDNI SITI NURMILA</t>
-  </si>
-  <si>
-    <t>19,9</t>
-  </si>
-  <si>
-    <t>44,1</t>
-  </si>
-  <si>
-    <t>41,5</t>
-  </si>
-  <si>
-    <t>52,9</t>
-  </si>
-  <si>
-    <t>29,1</t>
-  </si>
-  <si>
-    <t>40,1</t>
-  </si>
-  <si>
-    <t>38,3</t>
-  </si>
-  <si>
-    <t>29,5</t>
-  </si>
-  <si>
-    <t>20,4</t>
-  </si>
-  <si>
-    <t>33,2</t>
-  </si>
-  <si>
-    <t>38,7</t>
-  </si>
-  <si>
-    <t>kurang</t>
-  </si>
-  <si>
-    <t>baik</t>
+    <t>AZWA NURFAISAL</t>
+  </si>
+  <si>
+    <t>DIANA AQILA PUTRI</t>
+  </si>
+  <si>
+    <t>MUHAMAD BAYU ANUGRAH</t>
+  </si>
+  <si>
+    <t>MUHAMMAD IKBAR MAULADIN</t>
+  </si>
+  <si>
+    <t>RAFAEL ARSYIL ARRAHMAN</t>
+  </si>
+  <si>
+    <t>RAPITA ROSMAYANTI</t>
+  </si>
+  <si>
+    <t>SITI NAILA AZZAHRA</t>
+  </si>
+  <si>
+    <t>KURANG</t>
+  </si>
+  <si>
+    <t>BAIK</t>
+  </si>
+  <si>
+    <t>LEBIH</t>
+  </si>
+  <si>
+    <t>OBESITAS</t>
   </si>
 </sst>
 </file>
@@ -601,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B65EA9BD-8D15-44AC-94E5-ABF90C086641}">
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="25.109375" customWidth="1"/>
@@ -673,14 +625,14 @@
       <c r="B2">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>34</v>
+      <c r="C2" s="2">
+        <v>37</v>
       </c>
       <c r="D2" s="2">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F2" s="3">
         <v>80</v>
@@ -689,7 +641,7 @@
         <v>50</v>
       </c>
       <c r="H2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" s="6">
         <v>1</v>
@@ -732,14 +684,14 @@
       <c r="B3">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>35</v>
+      <c r="C3" s="2">
+        <v>38</v>
       </c>
       <c r="D3" s="2">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="F3" s="3">
         <v>90</v>
@@ -748,7 +700,7 @@
         <v>60</v>
       </c>
       <c r="H3" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I3" s="6">
         <v>1</v>
@@ -791,23 +743,23 @@
       <c r="B4">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>36</v>
+      <c r="C4" s="2">
+        <v>44</v>
       </c>
       <c r="D4" s="2">
-        <v>153</v>
+        <v>126</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F4" s="3">
         <v>90</v>
       </c>
       <c r="G4" s="4">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H4" s="5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4" s="6">
         <v>1</v>
@@ -851,22 +803,22 @@
         <v>6</v>
       </c>
       <c r="C5" s="2">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" s="2">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="E5" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F5" s="3">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="G5" s="4">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H5" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I5" s="6">
         <v>1</v>
@@ -910,22 +862,22 @@
         <v>6</v>
       </c>
       <c r="C6" s="2">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="D6" s="2">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
       <c r="F6" s="3">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="G6" s="4">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H6" s="5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I6" s="6">
         <v>1</v>
@@ -969,25 +921,25 @@
         <v>6</v>
       </c>
       <c r="C7" s="2">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="D7" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="F7" s="3">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G7" s="4">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H7" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6">
         <v>1</v>
@@ -1027,26 +979,26 @@
       <c r="B8">
         <v>6</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>37</v>
+      <c r="C8" s="2">
+        <v>30</v>
       </c>
       <c r="D8" s="2">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="E8" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="F8" s="3">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="G8" s="4">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="H8" s="5">
         <v>2</v>
       </c>
       <c r="I8" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" s="6">
         <v>1</v>
@@ -1080,476 +1032,137 @@
       </c>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9">
-        <v>6</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="2">
-        <v>137</v>
-      </c>
-      <c r="E9" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" s="3">
-        <v>85</v>
-      </c>
-      <c r="G9" s="4">
-        <v>50</v>
-      </c>
-      <c r="H9" s="5">
-        <v>2</v>
-      </c>
-      <c r="I9" s="6">
-        <v>1</v>
-      </c>
-      <c r="J9" s="6">
-        <v>1</v>
-      </c>
-      <c r="K9" s="6">
-        <v>1</v>
-      </c>
-      <c r="L9" s="6">
-        <v>1</v>
-      </c>
-      <c r="M9" s="6">
-        <v>1</v>
-      </c>
-      <c r="N9" s="6">
-        <v>1</v>
-      </c>
-      <c r="O9" s="6">
-        <v>1</v>
-      </c>
-      <c r="P9" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="6">
-        <v>1</v>
-      </c>
-      <c r="R9" s="6">
-        <v>1</v>
-      </c>
-      <c r="S9" s="6">
-        <v>1</v>
-      </c>
+      <c r="A9" s="1"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
     </row>
     <row r="10" spans="1:19">
-      <c r="A10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10">
-        <v>6</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" s="2">
-        <v>141</v>
-      </c>
-      <c r="E10" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" s="3">
-        <v>90</v>
-      </c>
-      <c r="G10" s="4">
-        <v>70</v>
-      </c>
-      <c r="H10" s="5">
-        <v>1</v>
-      </c>
-      <c r="I10" s="6">
-        <v>1</v>
-      </c>
-      <c r="J10" s="6">
-        <v>1</v>
-      </c>
-      <c r="K10" s="6">
-        <v>1</v>
-      </c>
-      <c r="L10" s="6">
-        <v>1</v>
-      </c>
-      <c r="M10" s="6">
-        <v>1</v>
-      </c>
-      <c r="N10" s="6">
-        <v>1</v>
-      </c>
-      <c r="O10" s="6">
-        <v>1</v>
-      </c>
-      <c r="P10" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="6">
-        <v>1</v>
-      </c>
-      <c r="R10" s="6">
-        <v>1</v>
-      </c>
-      <c r="S10" s="6">
-        <v>1</v>
-      </c>
+      <c r="A10" s="1"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
     </row>
     <row r="11" spans="1:19">
-      <c r="A11" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11">
-        <v>6</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" s="2">
-        <v>139</v>
-      </c>
-      <c r="E11" t="s">
-        <v>46</v>
-      </c>
-      <c r="F11" s="3">
-        <v>90</v>
-      </c>
-      <c r="G11" s="4">
-        <v>60</v>
-      </c>
-      <c r="H11" s="5">
-        <v>0</v>
-      </c>
-      <c r="I11" s="6">
-        <v>1</v>
-      </c>
-      <c r="J11" s="6">
-        <v>1</v>
-      </c>
-      <c r="K11" s="6">
-        <v>1</v>
-      </c>
-      <c r="L11" s="6">
-        <v>1</v>
-      </c>
-      <c r="M11" s="6">
-        <v>1</v>
-      </c>
-      <c r="N11" s="6">
-        <v>1</v>
-      </c>
-      <c r="O11" s="6">
-        <v>1</v>
-      </c>
-      <c r="P11" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q11" s="6">
-        <v>1</v>
-      </c>
-      <c r="R11" s="6">
-        <v>1</v>
-      </c>
-      <c r="S11" s="6">
-        <v>1</v>
-      </c>
+      <c r="A11" s="1"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
     </row>
     <row r="12" spans="1:19">
-      <c r="A12" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12">
-        <v>6</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="2">
-        <v>145</v>
-      </c>
-      <c r="E12" t="s">
-        <v>45</v>
-      </c>
-      <c r="F12" s="3">
-        <v>90</v>
-      </c>
-      <c r="G12" s="4">
-        <v>60</v>
-      </c>
-      <c r="H12" s="5">
-        <v>3</v>
-      </c>
-      <c r="I12" s="6">
-        <v>1</v>
-      </c>
-      <c r="J12" s="6">
-        <v>1</v>
-      </c>
-      <c r="K12" s="6">
-        <v>1</v>
-      </c>
-      <c r="L12" s="6">
-        <v>2</v>
-      </c>
-      <c r="M12" s="6">
-        <v>1</v>
-      </c>
-      <c r="N12" s="6">
-        <v>1</v>
-      </c>
-      <c r="O12" s="6">
-        <v>1</v>
-      </c>
-      <c r="P12" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="6">
-        <v>1</v>
-      </c>
-      <c r="R12" s="6">
-        <v>1</v>
-      </c>
-      <c r="S12" s="6">
-        <v>1</v>
-      </c>
+      <c r="A12" s="1"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
     </row>
     <row r="13" spans="1:19">
-      <c r="A13" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13">
-        <v>6</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="2">
-        <v>140</v>
-      </c>
-      <c r="E13" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="3">
-        <v>100</v>
-      </c>
-      <c r="G13" s="4">
-        <v>70</v>
-      </c>
-      <c r="H13" s="5">
-        <v>2</v>
-      </c>
-      <c r="I13" s="6">
-        <v>1</v>
-      </c>
-      <c r="J13" s="6">
-        <v>1</v>
-      </c>
-      <c r="K13" s="6">
-        <v>2</v>
-      </c>
-      <c r="L13" s="6">
-        <v>1</v>
-      </c>
-      <c r="M13" s="6">
-        <v>1</v>
-      </c>
-      <c r="N13" s="6">
-        <v>1</v>
-      </c>
-      <c r="O13" s="6">
-        <v>1</v>
-      </c>
-      <c r="P13" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="6">
-        <v>1</v>
-      </c>
-      <c r="R13" s="6">
-        <v>1</v>
-      </c>
-      <c r="S13" s="6">
-        <v>1</v>
-      </c>
+      <c r="A13" s="1"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
     </row>
     <row r="14" spans="1:19">
-      <c r="A14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14">
-        <v>6</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="2">
-        <v>147</v>
-      </c>
-      <c r="E14" t="s">
-        <v>46</v>
-      </c>
-      <c r="F14" s="3">
-        <v>100</v>
-      </c>
-      <c r="G14" s="4">
-        <v>70</v>
-      </c>
-      <c r="H14" s="5">
-        <v>4</v>
-      </c>
-      <c r="I14" s="6">
-        <v>1</v>
-      </c>
-      <c r="J14" s="6">
-        <v>1</v>
-      </c>
-      <c r="K14" s="6">
-        <v>1</v>
-      </c>
-      <c r="L14" s="6">
-        <v>1</v>
-      </c>
-      <c r="M14" s="6">
-        <v>1</v>
-      </c>
-      <c r="N14" s="6">
-        <v>1</v>
-      </c>
-      <c r="O14" s="6">
-        <v>1</v>
-      </c>
-      <c r="P14" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="6">
-        <v>1</v>
-      </c>
-      <c r="R14" s="6">
-        <v>1</v>
-      </c>
-      <c r="S14" s="6">
-        <v>1</v>
-      </c>
+      <c r="A14" s="1"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
     </row>
     <row r="15" spans="1:19">
-      <c r="A15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15">
-        <v>6</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="2">
-        <v>150</v>
-      </c>
-      <c r="E15" t="s">
-        <v>45</v>
-      </c>
-      <c r="F15" s="3">
-        <v>88</v>
-      </c>
-      <c r="G15" s="4">
-        <v>50</v>
-      </c>
-      <c r="H15" s="5">
-        <v>3</v>
-      </c>
-      <c r="I15" s="6">
-        <v>1</v>
-      </c>
-      <c r="J15" s="6">
-        <v>1</v>
-      </c>
-      <c r="K15" s="6">
-        <v>1</v>
-      </c>
-      <c r="L15" s="6">
-        <v>1</v>
-      </c>
-      <c r="M15" s="6">
-        <v>1</v>
-      </c>
-      <c r="N15" s="6">
-        <v>1</v>
-      </c>
-      <c r="O15" s="6">
-        <v>1</v>
-      </c>
-      <c r="P15" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="6">
-        <v>1</v>
-      </c>
-      <c r="R15" s="6">
-        <v>1</v>
-      </c>
-      <c r="S15" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19">
-      <c r="A16" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16">
-        <v>6</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" s="2">
-        <v>149</v>
-      </c>
-      <c r="E16" t="s">
-        <v>45</v>
-      </c>
-      <c r="F16" s="3">
-        <v>90</v>
-      </c>
-      <c r="G16" s="4">
-        <v>60</v>
-      </c>
-      <c r="H16" s="7">
-        <v>0</v>
-      </c>
-      <c r="I16" s="6">
-        <v>1</v>
-      </c>
-      <c r="J16" s="6">
-        <v>1</v>
-      </c>
-      <c r="K16" s="6">
-        <v>1</v>
-      </c>
-      <c r="L16" s="6">
-        <v>1</v>
-      </c>
-      <c r="M16" s="6">
-        <v>1</v>
-      </c>
-      <c r="N16" s="6">
-        <v>1</v>
-      </c>
-      <c r="O16" s="6">
-        <v>1</v>
-      </c>
-      <c r="P16" s="6">
-        <v>1</v>
-      </c>
-      <c r="Q16" s="6">
-        <v>1</v>
-      </c>
-      <c r="R16" s="6">
-        <v>1</v>
-      </c>
-      <c r="S16" s="6">
-        <v>1</v>
-      </c>
+      <c r="A15" s="1"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>